<commit_message>
fix: Runway avg IFERROR + Burn Rate excludes aportes
- Runway Média Mensal: IFERROR wrapper so AVERAGE of 'N/A' text
  shows 'N/A' instead of #DIV/0! error
- Burn Rate formula: =-(FCO + Rec.Fin) instead of =-Variação,
  excluding aportes/estornos as per plan description
</commit_message>
<xml_diff>
--- a/Nuvio_Tech_Corrigida.xlsx
+++ b/Nuvio_Tech_Corrigida.xlsx
@@ -23147,15 +23147,15 @@
         </is>
       </c>
       <c r="B17" s="6">
-        <f>-B14</f>
+        <f>-(B7+B10)</f>
         <v/>
       </c>
       <c r="C17" s="6">
-        <f>-C14</f>
+        <f>-(C7+C10)</f>
         <v/>
       </c>
       <c r="D17" s="6">
-        <f>-D14</f>
+        <f>-(D7+D10)</f>
         <v/>
       </c>
       <c r="E17" s="6">
@@ -23186,8 +23186,8 @@
         <f>IF(D17&lt;=0,"N/A",D15/D17)</f>
         <v/>
       </c>
-      <c r="E18" s="6">
-        <f>AVERAGE(B18:D18)</f>
+      <c r="E18" s="18">
+        <f>IFERROR(AVERAGE(B18:D18),"N/A")</f>
         <v/>
       </c>
       <c r="F18" s="14" t="inlineStr">

</xml_diff>